<commit_message>
Add excel xlsx read write, html render to pdf for webpdf, add image module, replace qrcode, add async_send_email, refactor the markdown2html module
</commit_message>
<xml_diff>
--- a/docs/kk_out.xlsx
+++ b/docs/kk_out.xlsx
@@ -23,6 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
   <fonts count="8">
     <font>
       <sz val="10"/>
@@ -91,8 +94,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="4">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -288,7 +296,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -298,7 +306,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C4" t="s">

</xml_diff>

<commit_message>
Change pzexcel pzword to cmake .. -DENABLE_OFFICE=ON
</commit_message>
<xml_diff>
--- a/docs/kk_out.xlsx
+++ b/docs/kk_out.xlsx
@@ -315,10 +315,10 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>999.804000</v>
+        <v>999.804</v>
       </c>
       <c r="B5">
-        <v>443888.567890</v>
+        <v>443888.56789</v>
       </c>
     </row>
   </sheetData>

</xml_diff>